<commit_message>
Clarify dialogue answers in English workbook notes
</commit_message>
<xml_diff>
--- a/Studymaterials/中学生英作文be動詞現在形編.xlsx
+++ b/Studymaterials/中学生英作文be動詞現在形編.xlsx
@@ -421,7 +421,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -489,6 +489,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -933,10 +936,11 @@
       <c r="I3" s="25" t="n"/>
       <c r="J3" s="26" t="n"/>
     </row>
-    <row r="4" ht="18" customHeight="1" s="6">
+    <row r="4" ht="36" customHeight="1" s="6">
       <c r="A4" s="20" t="inlineStr">
         <is>
-          <t>※短縮形が2つあるところは、短縮形1と短縮形2の順番が逆でも正解です。</t>
+          <t>※短縮形が2つあるところは、短縮形1と短縮形2の順番が逆でも正解です。
+※相手が答える形なので、返答では I / we ではなく you を使います。</t>
         </is>
       </c>
       <c r="B4" s="27" t="n"/>
@@ -2021,10 +2025,11 @@
       <c r="I72" s="25" t="n"/>
       <c r="J72" s="26" t="n"/>
     </row>
-    <row r="73" ht="18" customHeight="1" s="6">
+    <row r="73" ht="36" customHeight="1" s="6">
       <c r="A73" s="20" t="inlineStr">
         <is>
-          <t>※短縮形が2つあるところは、短縮形1と短縮形2の順番が逆でも正解です。</t>
+          <t>※短縮形が2つあるところは、短縮形1と短縮形2の順番が逆でも正解です。
+※相手が答える形なので、返答では I / we ではなく you を使います。</t>
         </is>
       </c>
       <c r="B73" s="27" t="n"/>
@@ -3487,8 +3492,8 @@
     <mergeCell ref="A113:J113"/>
     <mergeCell ref="A71:J71"/>
   </mergeCells>
-  <printOptions horizontalCentered="1" verticalCentered="0" gridLines="1"/>
-  <pageMargins left="0.25" right="0.25" top="0.2" bottom="0.2" header="0.1" footer="0.1"/>
+  <printOptions horizontalCentered="1" verticalCentered="1" gridLines="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.1" footer="0.1"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1" verticalDpi="0"/>
   <rowBreaks count="4" manualBreakCount="4">
     <brk id="35" min="0" max="16383" man="1"/>
@@ -3552,10 +3557,11 @@
       <c r="I3" s="25" t="n"/>
       <c r="J3" s="26" t="n"/>
     </row>
-    <row r="4" ht="18" customHeight="1" s="6">
+    <row r="4" ht="36" customHeight="1" s="6">
       <c r="A4" s="20" t="inlineStr">
         <is>
-          <t>※短縮形が2つあるところは、短縮形1と短縮形2の順番が逆でも正解です。</t>
+          <t>※短縮形が2つあるところは、短縮形1と短縮形2の順番が逆でも正解です。
+※相手が答える形なので、返答では I / we ではなく you を使います。</t>
         </is>
       </c>
       <c r="B4" s="27" t="n"/>
@@ -3715,7 +3721,7 @@
     <row r="14" ht="26" customHeight="1" s="6">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>正解（返答）：Yes, I am.</t>
+          <t>正解（返答）：Yes, you are.</t>
         </is>
       </c>
       <c r="B14" s="27" t="n"/>
@@ -3747,7 +3753,7 @@
     <row r="16" ht="26" customHeight="1" s="6">
       <c r="A16" s="21" t="inlineStr">
         <is>
-          <t>正解（基本形）：No, I am not.</t>
+          <t>正解（基本形）：No, you are not.</t>
         </is>
       </c>
       <c r="B16" s="27" t="n"/>
@@ -3763,7 +3769,7 @@
     <row r="17" ht="26" customHeight="1" s="6">
       <c r="A17" s="21" t="inlineStr">
         <is>
-          <t>正解（短縮形）：No, I'm not.</t>
+          <t>正解（短縮形）：No, you aren't.</t>
         </is>
       </c>
       <c r="B17" s="27" t="n"/>
@@ -4640,10 +4646,11 @@
       <c r="I72" s="25" t="n"/>
       <c r="J72" s="26" t="n"/>
     </row>
-    <row r="73" ht="18" customHeight="1" s="6">
+    <row r="73" ht="36" customHeight="1" s="6">
       <c r="A73" s="20" t="inlineStr">
         <is>
-          <t>※短縮形が2つあるところは、短縮形1と短縮形2の順番が逆でも正解です。</t>
+          <t>※短縮形が2つあるところは、短縮形1と短縮形2の順番が逆でも正解です。
+※相手が答える形なので、返答では I / we ではなく you を使います。</t>
         </is>
       </c>
       <c r="B73" s="27" t="n"/>
@@ -4819,7 +4826,7 @@
     <row r="84" ht="26" customHeight="1" s="6">
       <c r="A84" s="21" t="inlineStr">
         <is>
-          <t>正解（返答）：Yes, we are.</t>
+          <t>正解（返答）：Yes, you are.</t>
         </is>
       </c>
       <c r="B84" s="27" t="n"/>
@@ -4851,7 +4858,7 @@
     <row r="86" ht="26" customHeight="1" s="6">
       <c r="A86" s="21" t="inlineStr">
         <is>
-          <t>正解（基本形）：No, we are not.</t>
+          <t>正解（基本形）：No, you are not.</t>
         </is>
       </c>
       <c r="B86" s="27" t="n"/>
@@ -4867,7 +4874,7 @@
     <row r="87" ht="26" customHeight="1" s="6">
       <c r="A87" s="21" t="inlineStr">
         <is>
-          <t>正解（短縮形1）：No, we aren't.</t>
+          <t>正解（短縮形1）：No, you aren't.</t>
         </is>
       </c>
       <c r="B87" s="27" t="n"/>
@@ -4883,7 +4890,7 @@
     <row r="88" ht="26" customHeight="1" s="6">
       <c r="A88" s="21" t="inlineStr">
         <is>
-          <t>正解（短縮形2）：No, we're not.</t>
+          <t>正解（短縮形2）：No, you're not.</t>
         </is>
       </c>
       <c r="B88" s="27" t="n"/>
@@ -6106,8 +6113,8 @@
     <mergeCell ref="A113:J113"/>
     <mergeCell ref="A71:J71"/>
   </mergeCells>
-  <printOptions horizontalCentered="1" verticalCentered="0" gridLines="1"/>
-  <pageMargins left="0.25" right="0.25" top="0.2" bottom="0.2" header="0.1" footer="0.1"/>
+  <printOptions horizontalCentered="1" verticalCentered="1" gridLines="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.1" footer="0.1"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1" verticalDpi="0"/>
   <rowBreaks count="4" manualBreakCount="4">
     <brk id="35" min="0" max="16383" man="1"/>

</xml_diff>